<commit_message>
Implement SOSA-next crosswalk dispositions
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -378,14 +378,9 @@
           <t>sosa:ActuatingProcedure</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>rdfs:subClassOf</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>sosa:Procedure and (cco:prescribes some sosa:Actuation)</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Remove the cco:prescribes restriction and rely on the native ActuatingProcedure subClassOf Procedure hierarchy. The source definition supports the specialization: an ActuatingProcedure specifies how to make an Actuation. The current existential nevertheless entails an actual Actuation, while the external universal over the broad CCO prescribes relation would require every entity for which the directive serves as a rule, guide, or model to be an Actuation. Neither CCO restriction safely expresses the source specialization.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -451,7 +446,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>bfo:MaterialEntity and (bfo:bearer_of some (bfo:RealizableEntity and (bfo:has_realization some sosa:Actuation))) and (cco:agent_in some sosa:Actuation)</t>
+          <t>bfo:MaterialEntity</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Replace the current composite subclass mapping with sosa:Actuator rdfs:subClassOf bfo:MaterialEntity. Remove the bearer_of, has_realization, and agent_in existential restrictions. This preserves the project's deliberate materiality commitment without requiring an actual Actuation.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -468,12 +468,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>owl:equivalentClass</t>
+          <t>rdfs:subClassOf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cco:PlannedAct and (sosa:deployedSystem some sosa:System) and (sosa:deployedOnPlatform some bfo:MaterialEntity)</t>
+          <t>cco:PlannedAct and (sosa:deployedAsset some sosa:Asset)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Replace the current equivalent-class mapping with sosa:Deployment rdfs:subClassOf cco:PlannedAct and (sosa:deployedAsset some sosa:Asset). The source defines a Deployment as an arrangement of one or more Assets and states that it may involve Platforms, Systems, or both. The current mandatory System and Platform restrictions are therefore too narrow. A one-way subclass is retained because the source supports these as necessary conditions but does not justify the reverse classification of every matching PlannedAct as a Deployment.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -539,7 +544,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>bfo:Entity and (sosa:isFeatureOfInterestOf some (sosa:Observation or sosa:Sampling or sosa:Actuation))</t>
+          <t>bfo:Entity and (sosa:isFeatureOfInterestOf some (sosa:Execution or sosa:ExecutionCollection or sosa:Deployment))</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Widen the current equivalent-class filler from Observation-or-Sampling-or-Actuation to Execution-or-ExecutionCollection-or-Deployment. This matches the exact pinned isFeatureOfInterestOf signature: the narrower execution classes are already subclasses of Execution, and their collection classes are subclasses of ExecutionCollection.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -576,14 +586,9 @@
           <t>sosa:Observation</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>rdfs:subClassOf</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>cco:PlannedAct and (cco:has_process_part some (cco:ActOfMeasuring and cco:ActOfObservation))</t>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Remove the direct Observation mapping row. Observation is already a native subclass of Execution and therefore inherits the governed Execution-to-PlannedAct mapping. The additional process-part restriction is unsupported: CCO ActOfObservation requires sense-based acquisition, while SOSA includes automated observations, and SOSA's broader estimation and calculation scope does not require every Observation to contain a distinct CCO ActOfMeasuring process part.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -620,14 +625,9 @@
           <t>sosa:ObservingProcedure</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>rdfs:subClassOf</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>sosa:Procedure and (cco:prescribes some sosa:Observation)</t>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Remove the cco:prescribes restriction and rely on the native ObservingProcedure subClassOf Procedure hierarchy. The source definition supports the specialization: an ObservingProcedure specifies how to make an Observation. The current existential nevertheless entails an actual Observation, while the external universal over the broad CCO prescribes relation would require every entity for which the directive serves as a rule, guide, or model to be an Observation. Neither CCO restriction safely expresses the source specialization.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -649,7 +649,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>bfo:MaterialEntity and (sosa:hosts some sosa:System)</t>
+          <t>sosa:Asset and bfo:MaterialEntity and (sosa:hosts some sosa:Asset)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Replace the current equivalence with sosa:Platform owl:equivalentClass sosa:Asset and bfo:MaterialEntity and (sosa:hosts some sosa:Asset). The pinned definition characterizes a Platform as an Asset that hosts other Assets, particularly Systems and Platforms; the external System-or-Platform filler is therefore still too narrow. The MaterialEntity conjunct preserves the project's existing materiality commitment.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -671,7 +676,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>cco:DirectiveInformationContentEntity and (cco:prescribes some bfo:Process)</t>
+          <t>cco:DirectiveInformationContentEntity</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Replace the current composite mapping with the single axiom sosa:Procedure rdfs:subClassOf cco:DirectiveInformationContentEntity. The exact pinned target is cco:ont00000965, labelled Directive Information Content Entity, not Prescriptive Information Content Entity. Remove the additional cco:prescribes some bfo:Process restriction because the source definition does not require every reusable Procedure to prescribe an actual Process. The weaker existential inherited from the CCO target's own definition remains.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -688,12 +698,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>owl:equivalentClass</t>
+          <t>rdfs:subClassOf</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>(bfo:SpecificallyDependentContinuant or bfo:ProcessProfile)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Weaken the current equivalence to sosa:Property rdfs:subClassOf (bfo:SpecificallyDependentContinuant or bfo:ProcessProfile). The two-branch union remains the project's necessary upper bound for continuant and occurrent properties, but the reverse implications are unsupported: not every specifically dependent continuant or process profile is a SOSA Property.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -737,7 +752,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>bfo:ObjectAggregate and (bfo:has_member_part some (sosa:Sample or sosa:SampleCollection))</t>
+          <t>bfo:Continuant and (bfo:has_continuant_part some (sosa:Sample or sosa:SampleCollection))</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Adopt the external corrected mapping: sosa:SampleCollection rdfs:subClassOf bfo:Continuant and (bfo:has_continuant_part some (sosa:Sample or sosa:SampleCollection)). This removes the material-only ObjectAggregate and has_member_part commitments while retaining an existential continuant-parthood interpretation for at least one Sample or nested SampleCollection. This is a deliberate project-level formalization of SOSA collection membership; no universal parthood restriction is asserted.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -754,12 +774,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>owl:equivalentClass</t>
+          <t>rdfs:subClassOf</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>bfo:MaterialEntity and (bfo:bearer_of some (bfo:RealizableEntity and (bfo:has_realization some sosa:Sampling))) and (cco:agent_in some sosa:Sampling)</t>
+          <t>bfo:MaterialEntity</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Replace the current equivalent-class mapping with sosa:Sampler rdfs:subClassOf bfo:MaterialEntity. Remove the reverse implication and the bearer_of, has_realization, and agent_in existential restrictions. This preserves the project's deliberate materiality commitment without requiring an actual Sampling.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -818,14 +843,9 @@
           <t>sosa:SamplingProcedure</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>rdfs:subClassOf</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>sosa:Procedure and (cco:prescribes some sosa:Sampling)</t>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Remove the cco:prescribes restriction and rely on the native SamplingProcedure subClassOf Procedure hierarchy. The source definition supports the specialization: a SamplingProcedure specifies how to make a Sampling. The current existential nevertheless entails an actual Sampling, while the external universal over the broad CCO prescribes relation would require every entity for which the directive serves as a rule, guide, or model to be a Sampling. Neither CCO restriction safely expresses the source specialization.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -857,14 +877,9 @@
           <t>sosa:SpatialSample</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>rdfs:subClassOf</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>sosa:Sample and (sosa:isSampleOf some (bfo:Entity and (bfo:occupies_spatial_region some bfo:SpatialRegion)))</t>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Remove the active cross-ontology restriction and retain the native SpatialSample subClassOf Sample axiom. The source defines spatiality through the sample's own location and shape. Neither requiring the represented FeatureOfInterest to occupy a spatial region nor requiring production by a Sampling whose FeatureOfInterest occupies a spatial region captures that defining condition.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -903,12 +918,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>owl:equivalentClass</t>
+          <t>rdfs:subClassOf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>cco:Cause and (cco:is_cause_of some sosa:Observation)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Replace the equivalent-class axiom with a one-way subclass axiom. Every SOSA Stimulus may be modeled as a CCO Cause that is cause of some Observation, but not every cause of an Observation is thereby a SOSA Stimulus.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1175,14 +1195,9 @@
           <t>sosa:hasOperatingConditions</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>owl:propertyChainAxiom</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>bfo:bearer_of o cco:is_subject_of</t>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>The chain bfo:bearer_of o cco:is_subject_of concludes in an Information Content Entity, whereas the SOSA-next relation ranges over OperatingConditions, Observation, or ObservationCollection. The chain does not express the source relation.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1197,14 +1212,9 @@
           <t>sosa:hasSystemCapability</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>owl:propertyChainAxiom</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>bfo:bearer_of o cco:is_subject_of</t>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>The chain bfo:bearer_of o cco:is_subject_of concludes in an Information Content Entity, whereas the SOSA-next relation ranges over Observation or ObservationCollection. The chain does not express the source relation.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1335,14 +1345,9 @@
           <t>sosa:actsOn</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>bfo:has_participant</t>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>The source relation has an Actuator subject, whereas bfo:has_participant has a process domain. The current subproperty axiom can therefore classify an actuator as a process.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1357,14 +1362,9 @@
           <t>sosa:actsOnProperty</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>cco:affects</t>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>cco:affects has a continuant range, whereas sosa:Property includes the ProcessProfile branch. The current mapping can therefore impose continuant typing on an occurrent property.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1467,14 +1467,9 @@
           <t>sosa:featureHasUltimateSample</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>cco:is_output_of</t>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Remove the cco:is_output_of superproperty. The source relation runs from a FeatureOfInterest to an ultimate Sample or SampleCollection. It does not relate a Continuant output to the Sampling process that produced it. The current mapping would instead place the source and target into the CCO output-to-process signature.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1489,14 +1484,9 @@
           <t>sosa:forProperty</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>owl:propertyChainAxiom</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>cco:described_by o cco:is_about</t>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>The chain cco:described_by o cco:is_about captures an entity being described by information that is about a property. It does not establish that the entity acts on or observes that property, which is the intended meaning of sosa:forProperty. This semantic mismatch applies regardless of the CCO version.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1518,7 +1508,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>cco:is_output_of</t>
+          <t>bfo:participates_in</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Replace the current cco:is_output_of superproperty with bfo:participates_in. The source relation is inverse to sosa:deployedAsset, whose governed mapping is under bfo:has_participant; participates_in is the corresponding inverse direction.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1545,14 +1540,9 @@
           <t>sosa:hasInput</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>cco:has_input</t>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Remove the cco:has_input superproperty. The source relation runs from a Procedure, which is mapped as a prescriptive information content entity, whereas CCO has_input has a Process domain. No direct CCO superproperty expresses a Procedure-to-required-input-specification relation.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1567,14 +1557,9 @@
           <t>sosa:hasInputValue</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>cco:has_input</t>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Remove the cco:has_input superproperty. Although the source subject is an Execution or ExecutionCollection, SOSA only states that the object assigns a value to an input used in the execution. It does not entail the stronger CCO condition that the object is a Continuant whose presence at the beginning is necessary for the Process to start.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1601,14 +1586,9 @@
           <t>sosa:hasOriginalSample</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>cco:is_output_of</t>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Remove the cco:is_output_of superproperty. The source relation runs from one Sample to another Sample identified as its original. It does not relate an output to the Sampling process that produced it, and the CCO mapping would incorrectly type the target Sample as a Process.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1623,14 +1603,9 @@
           <t>sosa:hasOutput</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>cco:is_output_of</t>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Remove the cco:is_output_of superproperty. The source relation runs from a Procedure to an output specification, while is_output_of runs from a Continuant output to the Process that produced it. A Procedure is not that process, and the current mapping also reverses the relation.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1688,7 +1663,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>cco:is_output_of</t>
+          <t>cco:has_output</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Replace cco:is_output_of with cco:has_output. The SOSA relation runs from an Execution or ExecutionCollection to its result, matching the CCO Process-to-Continuant output direction. The current mapping uses the inverse direction.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1778,7 +1758,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>cco:prescribes o cco:agent_in</t>
+          <t>cco:prescribes o cco:has_agent</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Replace the misdirected chain with cco:prescribes o cco:has_agent. The pinned CCO confirms that prescribes is inverse to prescribed_by and has_agent is inverse to agent_in.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1800,7 +1785,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>cco:agent_in o cco:prescribes</t>
+          <t>cco:agent_in o cco:prescribed_by</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Replace the category-incompatible chain with cco:agent_in o cco:prescribed_by. This follows the path from a system through an execution in which it is an agent to the procedure prescribing that execution.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2225,14 +2215,9 @@
           <t>sosa:observedProperty</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>cco:has_input</t>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>cco:has_input has a continuant range, whereas sosa:Property includes the ProcessProfile branch. The current mapping can impose continuant typing on an occurrent property.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2247,14 +2232,9 @@
           <t>sosa:observes</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>rdfs:subPropertyOf</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>bfo:has_participant</t>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>The source relation has a Sensor subject, whereas bfo:has_participant has a process domain. The current subproperty axiom can therefore classify a sensor as a process.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2276,7 +2256,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>cco:process_starts</t>
+          <t>cco:is_cause_of</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Replace cco:process_starts with cco:is_cause_of. The source states that a Stimulus originated an Observation and thus supports causal direction from Stimulus to Observation, but does not establish the stronger temporal-start conditions required by cco:process_starts.</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2305,12 +2290,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>rdfs:range</t>
+          <t>rdfs:domain</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
           <t>bfo:TemporalRegion</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Replace the current rdfs:range bfo:TemporalRegion axiom with rdfs:domain bfo:TemporalRegion. The native inverse orientation runs from a temporal entity to an Execution or ExecutionCollection. No BFO or CCO temporal superproperty is adopted because the temporal entity is the time to which the result pertains, not necessarily the temporal region occupied by the Execution.</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2325,6 +2315,21 @@
           <t>sosa:phenomenonTime</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>rdfs:range</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>bfo:TemporalRegion</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Replace the explicitly unmapped disposition with rdfs:range bfo:TemporalRegion. The pinned source declares phenomenonTime as an owl:ObjectProperty from an Execution or ExecutionCollection to the time at which its result applies. No BFO or CCO temporal superproperty is adopted because this time may differ from the Execution's own occupied temporal region.</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr">
         <is>
           <t>urn:uuid:b311531a-d29f-4e0e-89f0-1f8341334eae</t>
@@ -2390,7 +2395,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>cco:is_about</t>
+          <t>cco:is_subject_of</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Replace cco:is_about with cco:is_subject_of. The source relation runs from an Observation or ObservationCollection to quality information pertaining to it. The Observation is therefore the subject of the InformationContentEntity; the inverse source relation qualityOf correctly maps to cco:is_about.</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2494,7 +2504,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>cco:process_started_by</t>
+          <t>cco:caused_by</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Replace cco:process_started_by with cco:caused_by. This is the inverse-side counterpart of adapting sosa:originated to cco:is_cause_of. The source supports Observation-to-Stimulus causal direction but does not entail the stronger temporal-start conditions of cco:process_started_by.</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">

</xml_diff>

<commit_message>
Complete SOSA-2023 mapping decisions
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -676,12 +676,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>cco:DirectiveInformationContentEntity</t>
+          <t>cco:ont00000965</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Replace the current composite mapping with the single axiom sosa:Procedure rdfs:subClassOf cco:DirectiveInformationContentEntity. The exact pinned target is cco:ont00000965, labelled Directive Information Content Entity, not Prescriptive Information Content Entity. Remove the additional cco:prescribes some bfo:Process restriction because the source definition does not require every reusable Procedure to prescribe an actual Process. The weaker existential inherited from the CCO target's own definition remains.</t>
+          <t>Map sosa:Procedure to the stable CCO class IRI cco:ont00000965. In the explicitly selected CCO target snapshot at upstream commit 010c99847a856e2fb70eb1b1b1287d19556c9290, this class is labelled Prescriptive Information Content Entity; the repository-wide current CCO dependency labels the same stable IRI Directive Information Content Entity. Using the canonical ont00000965 token avoids label-dependent resolution. Retain only the subclass mapping and no additional cco:prescribes some bfo:Process restriction because a reusable SOSA Procedure does not require an actually prescribed Process.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -860,9 +860,19 @@
           <t>sosa:Sensor</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>owl:equivalentClass</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>cco:Sensor</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Mapping deferred pending either the next CCO release or publication of the forthcoming SOSA 2023 Edition, because the required target category or alignment basis is not yet sufficiently stable.</t>
+          <t>Adopt the expert-crosswalk equivalence sosa:Sensor owl:equivalentClass cco:Sensor against the explicitly selected CCO development snapshot at upstream commit 010c99847a856e2fb70eb1b1b1287d19556c9290. In that snapshot cco:Sensor is equivalently characterized using a Material Entity bearing a Sensor Function or Sensor Role, matching the dispositional Sensor interpretation selected for this SOSA-2023 mapping track. The dependency is pinned by exact commit and SHA-256 and is not the repository-wide current SSN/SOSA CCO dependency.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1081,7 +1091,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Mapping not currently established; deferred pending further ontological analysis.</t>
+          <t>No additional direct BFO/CCO mapping is adopted. The pinned source already declares sosa:ActuatableProperty rdfs:subClassOf sosa:Property, so this class inherits the governed cross-ontology upper bound for sosa:Property without requiring a more specific BFO commitment.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1096,9 +1106,19 @@
           <t>sosa:Asset</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>rdfs:subClassOf</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>bfo:Continuant</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Mapping not currently established; deferred pending further ontological analysis.</t>
+          <t>Map sosa:Asset to bfo:Continuant as a weak upper-level placement. The pinned source defines an Asset as a resource involved in a Deployment and uses Asset as the superclass of System and Platform. The mapping does not assert a more specific BFO continuant subtype or the unsupported reverse implication.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1115,7 +1135,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Mapping not currently established; deferred pending further ontological analysis.</t>
+          <t>No additional direct BFO/CCO mapping is adopted. The pinned source already declares sosa:ObservableProperty rdfs:subClassOf sosa:Property, so this class inherits the governed cross-ontology upper bound for sosa:Property without requiring a more specific BFO commitment.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1132,7 +1152,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Mapping not currently established; deferred pending further ontological analysis.</t>
+          <t>No direct BFO/CCO class mapping is adopted. sosa:Result is deprecated in the SOSA 2023 Edition, and its broad outcome semantics do not justify a new cross-ontology class commitment. Result interoperability is handled through the governed result relations.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1729,14 +1749,9 @@
           <t>sosa:hosts</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>owl:propertyChainAxiom</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>bfo:bearer_of o bfo:has_realization o bfo:has_participant</t>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Remove the active BFO role-realization property-chain mapping. Although bfo:bearer_of o bfo:has_realization o bfo:has_participant is a valid OWL property chain, it can conclude sosa:hosts for arbitrary participants in a realization, which is broader than the SOSA hosts relation. Retain the native SOSA hosts semantics without a direct BFO/CCO mapping.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">

</xml_diff>

<commit_message>
Add SOSA-2023 mapping status metadata
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -335,14 +335,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="56" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="37.25" customHeight="1">
@@ -368,6 +369,11 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>coms:MappingStatus</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>coms:RowID</t>
         </is>
       </c>
@@ -385,6 +391,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>urn:uuid:11668420-475b-467e-ba23-7f96488ec7e2</t>
         </is>
       </c>
@@ -407,6 +418,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>urn:uuid:a4d06a9e-8e56-4199-86f5-82c2ea87766b</t>
         </is>
       </c>
@@ -429,6 +445,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>urn:uuid:31becfe4-ccc5-4100-a7c2-a59fe2f86b19</t>
         </is>
       </c>
@@ -456,6 +477,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>urn:uuid:dc44970b-082c-43c9-bf91-a3cec17e9e81</t>
         </is>
       </c>
@@ -483,6 +509,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>urn:uuid:e048daa4-a241-46b8-97ea-64aa13f58ae2</t>
         </is>
       </c>
@@ -505,6 +536,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>urn:uuid:31eb03df-4e8b-469b-b563-63679a5bf66b</t>
         </is>
       </c>
@@ -527,6 +563,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>urn:uuid:07060322-415d-4b32-baab-984fa77abbd6</t>
         </is>
       </c>
@@ -554,6 +595,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>urn:uuid:f7f210fc-b43d-4275-b122-0993282dc688</t>
         </is>
       </c>
@@ -576,6 +622,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>urn:uuid:7ea55b20-b2e9-4a97-abdc-13abb0eb4b9a</t>
         </is>
       </c>
@@ -593,6 +644,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>urn:uuid:3677c023-0651-4d65-9427-812b24cf7adb</t>
         </is>
       </c>
@@ -615,6 +671,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>urn:uuid:31d563c8-5d91-436e-b3a3-3170f8b4483a</t>
         </is>
       </c>
@@ -632,6 +693,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>urn:uuid:277e554b-faab-4405-a559-8d4f24993ea5</t>
         </is>
       </c>
@@ -659,6 +725,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>urn:uuid:59e7a370-d6ed-4046-905c-854752bf74cc</t>
         </is>
       </c>
@@ -686,6 +757,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>urn:uuid:ece2ea89-fff4-4cc1-9697-030c0a733353</t>
         </is>
       </c>
@@ -713,6 +789,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>urn:uuid:3feb0ec5-269e-41b4-865f-ca9437affcb2</t>
         </is>
       </c>
@@ -735,6 +816,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>urn:uuid:28402605-2ad7-4768-bd45-5aa87d293a5c</t>
         </is>
       </c>
@@ -762,6 +848,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>urn:uuid:83717e9f-ddd3-4f3e-8479-01838d8a654d</t>
         </is>
       </c>
@@ -789,6 +880,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>urn:uuid:d1d3c5cb-a3a5-4305-81b6-ed991ec62067</t>
         </is>
       </c>
@@ -811,6 +907,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>urn:uuid:f1852962-6094-4096-b9e5-45b2c81bc66b</t>
         </is>
       </c>
@@ -833,6 +934,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>urn:uuid:d4704d0a-a8cb-4ca0-a2a0-aa194de1ae21</t>
         </is>
       </c>
@@ -850,6 +956,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>urn:uuid:7dab14b2-c0ff-438e-bad2-074c25736c4d</t>
         </is>
       </c>
@@ -877,6 +988,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>urn:uuid:5c81ebfe-53f9-4173-a1c6-b1ee9986a660</t>
         </is>
       </c>
@@ -894,6 +1010,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>urn:uuid:2fd520df-df1a-43e4-935c-7ec033548d73</t>
         </is>
       </c>
@@ -916,6 +1037,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>urn:uuid:eef0b2ee-fc06-409d-b5b9-22f2cbdce3fb</t>
         </is>
       </c>
@@ -943,6 +1069,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>urn:uuid:2a1ddfd2-c95f-4d25-acd8-8856ef4166b5</t>
         </is>
       </c>
@@ -965,6 +1096,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>urn:uuid:73ddfafa-1d1f-4c25-a89a-0b8f04ba4940</t>
         </is>
       </c>
@@ -987,6 +1123,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>urn:uuid:2706ef81-3169-4ca8-9d38-8b683e9ebe01</t>
         </is>
       </c>
@@ -999,6 +1140,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>urn:uuid:25c98756-ede3-4fe3-8a74-e498011b0da9</t>
         </is>
       </c>
@@ -1011,6 +1157,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>urn:uuid:08fea714-bd84-4a7f-95d8-f37019c70c12</t>
         </is>
       </c>
@@ -1023,6 +1174,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>urn:uuid:c5a22b6f-d24d-451f-a9d3-ed3a46cb83b4</t>
         </is>
       </c>
@@ -1035,6 +1191,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>urn:uuid:b3961e11-66c4-406b-aef7-ec5425f0a1a9</t>
         </is>
       </c>
@@ -1057,6 +1218,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>urn:uuid:c66ea1c8-2d57-482c-b1ab-6ca82d6f8f90</t>
         </is>
       </c>
@@ -1079,6 +1245,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>urn:uuid:55b58986-6556-40f8-a521-6990f65a9729</t>
         </is>
       </c>
@@ -1096,6 +1267,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>urn:uuid:006f66b7-5f1a-432b-b9c0-1eb1d76b668f</t>
         </is>
       </c>
@@ -1123,6 +1299,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>urn:uuid:f04bd5ec-1d13-429c-a980-79310c2952d1</t>
         </is>
       </c>
@@ -1140,6 +1321,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>urn:uuid:16fc0c23-b688-4edd-959b-4617686f7650</t>
         </is>
       </c>
@@ -1156,6 +1342,11 @@
         </is>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t>urn:uuid:85ddba3d-797a-48fd-b52e-d9f04d206852</t>
         </is>
@@ -1172,14 +1363,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="56" customWidth="1" min="3" max="3"/>
     <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="37.25" customHeight="1">
@@ -1205,6 +1397,11 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>coms:MappingStatus</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>coms:RowID</t>
         </is>
       </c>
@@ -1222,6 +1419,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>urn:uuid:281bf661-130d-4508-9cfb-41640c74d565</t>
         </is>
       </c>
@@ -1239,6 +1441,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>urn:uuid:e8bea09c-9380-4f7d-9dbf-92b15095ac80</t>
         </is>
       </c>
@@ -1251,6 +1458,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>urn:uuid:1d7f918a-7c25-4c26-bb69-26072e2fac76</t>
         </is>
       </c>
@@ -1263,6 +1475,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>urn:uuid:edc8b7a0-fcd0-4dc7-a286-55218f6dc2c2</t>
         </is>
       </c>
@@ -1275,6 +1492,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>urn:uuid:d581367e-d0f4-491e-9d3e-ff1ac7655eee</t>
         </is>
       </c>
@@ -1287,6 +1509,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>urn:uuid:d69a7c8a-5f83-4924-aab6-33d6016fe06d</t>
         </is>
       </c>
@@ -1304,6 +1531,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>urn:uuid:ce089ac3-c908-47b9-9480-adba020cad7f</t>
         </is>
       </c>
@@ -1321,6 +1553,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>urn:uuid:af747b46-1967-4532-990f-02555c3d7a28</t>
         </is>
       </c>
@@ -1338,6 +1575,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>urn:uuid:26f5f739-2926-4f2c-b78b-35a28d56e7cc</t>
         </is>
       </c>
@@ -1355,6 +1597,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>urn:uuid:0dc53714-99d6-4219-95d4-fdeb832b6ea3</t>
         </is>
       </c>
@@ -1372,6 +1619,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>urn:uuid:96f8d18b-0491-41a4-b0d6-d7dde067b2e3</t>
         </is>
       </c>
@@ -1389,6 +1641,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>urn:uuid:27ce3724-23eb-4a3d-b2a1-e2615a139a81</t>
         </is>
       </c>
@@ -1411,6 +1668,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>urn:uuid:5d5f0473-515b-4ef3-b5d3-33e3027e7661</t>
         </is>
       </c>
@@ -1433,6 +1695,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>urn:uuid:55243300-5a36-4342-a089-79ec19b4574f</t>
         </is>
       </c>
@@ -1455,6 +1722,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>urn:uuid:0e7d7994-e6c4-4b2c-84e4-d91c8ec01255</t>
         </is>
       </c>
@@ -1477,6 +1749,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>urn:uuid:2d000038-5519-467a-8332-77ff24b2059e</t>
         </is>
       </c>
@@ -1494,6 +1771,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>urn:uuid:d53ed4f5-2351-416f-b104-b0bb251bf394</t>
         </is>
       </c>
@@ -1511,6 +1793,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>urn:uuid:58a661aa-3d05-4fe8-9146-4ed38f9bc29c</t>
         </is>
       </c>
@@ -1538,6 +1825,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>urn:uuid:ab8c2d57-82be-4344-9af8-74521d8d5568</t>
         </is>
       </c>
@@ -1550,6 +1842,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>urn:uuid:b1cd2525-4abc-46cd-bd1f-9f821161853a</t>
         </is>
       </c>
@@ -1567,6 +1864,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>urn:uuid:5c8026fc-c9ae-4fad-acdd-f722c23e960c</t>
         </is>
       </c>
@@ -1584,6 +1886,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>urn:uuid:a3919577-239e-493a-a137-1c7ec09b72ce</t>
         </is>
       </c>
@@ -1596,6 +1903,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>urn:uuid:cfed9d6b-3051-4a3b-824d-14cd3feda5b2</t>
         </is>
       </c>
@@ -1613,6 +1925,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>urn:uuid:772bd41b-1347-4b8d-a922-5cb5bb1ed716</t>
         </is>
       </c>
@@ -1630,6 +1947,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>urn:uuid:4f0b0675-329c-4588-9a51-c99793670972</t>
         </is>
       </c>
@@ -1642,6 +1964,11 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>urn:uuid:b19cbe47-53f4-4fc6-8175-136a215a98b5</t>
         </is>
       </c>
@@ -1654,6 +1981,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>urn:uuid:d3fe049a-dd1e-48fa-b0eb-63fe9fb61ddc</t>
         </is>
       </c>
@@ -1666,6 +1998,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>urn:uuid:95c48ef0-8b94-4cd8-b9b2-65110fad4aa3</t>
         </is>
       </c>
@@ -1693,6 +2030,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>urn:uuid:cc35e702-bfa0-42f7-b1a7-b3bd4cca6a76</t>
         </is>
       </c>
@@ -1705,6 +2047,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>urn:uuid:a2b2a51d-52d9-494a-a5c9-075c6f9204d4</t>
         </is>
       </c>
@@ -1727,6 +2074,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>urn:uuid:2dc7fa6c-e0e9-4ca6-8286-ba18786ed74b</t>
         </is>
       </c>
@@ -1739,6 +2091,11 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>urn:uuid:367c2d2e-a731-4300-a297-71daf3430fad</t>
         </is>
       </c>
@@ -1756,6 +2113,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>urn:uuid:d4d8448e-01ee-40e0-932e-a73ecd9c059b</t>
         </is>
       </c>
@@ -1783,6 +2145,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>urn:uuid:81a0efa2-c685-416e-95e5-470e4bb88f80</t>
         </is>
       </c>
@@ -1810,6 +2177,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>urn:uuid:f2800ed5-c34b-46a3-9128-141537c5e9b1</t>
         </is>
       </c>
@@ -1822,6 +2194,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>urn:uuid:065d887b-15b0-4489-9877-c0e2a2d46909</t>
         </is>
       </c>
@@ -1834,6 +2211,11 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>urn:uuid:5638dc4d-a0b4-4018-9ac5-c15a3e63ae1d</t>
         </is>
       </c>
@@ -1846,6 +2228,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>urn:uuid:2c1df02f-049f-4072-963d-b19a8a3237f0</t>
         </is>
       </c>
@@ -1858,6 +2245,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>urn:uuid:9ecbbdbb-c876-43c8-89b1-271ee720b45f</t>
         </is>
       </c>
@@ -1870,6 +2262,11 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>urn:uuid:2acbcdf8-1660-4463-89cb-f21f33a5b62c</t>
         </is>
       </c>
@@ -1882,6 +2279,11 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>urn:uuid:6ee83e53-abe6-40f8-b1e7-537c442514a4</t>
         </is>
       </c>
@@ -1894,6 +2296,11 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>urn:uuid:1be6a5bf-3543-4104-848f-e104a968cb8d</t>
         </is>
       </c>
@@ -1906,6 +2313,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>urn:uuid:7015fa54-a947-48bc-81cb-e7151a2e96f8</t>
         </is>
       </c>
@@ -1918,6 +2330,11 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>urn:uuid:9e9f40b7-1422-4c8f-97ba-b05621f046da</t>
         </is>
       </c>
@@ -1930,6 +2347,11 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>urn:uuid:555945fc-2a5e-4ad5-86cd-59c6a6a63f8a</t>
         </is>
       </c>
@@ -1942,6 +2364,11 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>urn:uuid:86247465-6a48-4a88-9e7e-10209bd3fe26</t>
         </is>
       </c>
@@ -1954,6 +2381,11 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>urn:uuid:fec60e9c-ae05-4bca-9f55-7f0fadee6f11</t>
         </is>
       </c>
@@ -1966,6 +2398,11 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t>urn:uuid:6da4ffeb-d979-46a6-af92-c7fb310ede52</t>
         </is>
       </c>
@@ -1978,6 +2415,11 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>urn:uuid:029d187d-bd5d-4d79-8283-f79cff4bf95c</t>
         </is>
       </c>
@@ -1990,6 +2432,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
           <t>urn:uuid:fbd6c485-44ea-43b8-b194-3ac490bf48fa</t>
         </is>
       </c>
@@ -2002,6 +2449,11 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
           <t>urn:uuid:32e5650f-da54-4941-a2ef-05d24c1ef00a</t>
         </is>
       </c>
@@ -2014,6 +2466,11 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
           <t>urn:uuid:12ccae61-a7e8-46ad-92f5-f8c703388176</t>
         </is>
       </c>
@@ -2026,6 +2483,11 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
           <t>urn:uuid:45f09d66-c0e2-43e3-909a-96b38e1116fc</t>
         </is>
       </c>
@@ -2038,6 +2500,11 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
           <t>urn:uuid:f813618d-5482-41c0-bc77-24a9ee34e2c8</t>
         </is>
       </c>
@@ -2050,6 +2517,11 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
           <t>urn:uuid:fb9c0a9e-d7bf-4fa5-97fe-3fe71ba5beaa</t>
         </is>
       </c>
@@ -2072,6 +2544,11 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
           <t>urn:uuid:a3bead3c-ca9a-42f8-bda5-176574fd71d0</t>
         </is>
       </c>
@@ -2094,6 +2571,11 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
           <t>urn:uuid:a83c6ba4-b0c0-43c5-9018-076120ab77e6</t>
         </is>
       </c>
@@ -2116,6 +2598,11 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
           <t>urn:uuid:45ab5b89-b48b-4472-b37a-e7a40271b340</t>
         </is>
       </c>
@@ -2138,6 +2625,11 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
           <t>urn:uuid:1db47c58-82e4-45ed-8c75-1daebdf9616b</t>
         </is>
       </c>
@@ -2160,6 +2652,11 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
           <t>urn:uuid:5f0b98b4-739e-45fa-b756-01f8e1a06566</t>
         </is>
       </c>
@@ -2172,6 +2669,11 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
           <t>urn:uuid:2a839a3f-02f3-47d8-8482-6960cf88625d</t>
         </is>
       </c>
@@ -2184,6 +2686,11 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
           <t>urn:uuid:1a74e4c4-7b3e-4538-9967-263dd3a7de90</t>
         </is>
       </c>
@@ -2196,6 +2703,11 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
           <t>urn:uuid:9a05a746-cc32-4d52-88d6-22da6833e880</t>
         </is>
       </c>
@@ -2208,6 +2720,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
           <t>urn:uuid:e69ea37a-e4dc-43d4-b90d-fe94d76da025</t>
         </is>
       </c>
@@ -2220,6 +2737,11 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
           <t>urn:uuid:81bb38b5-18d7-46fb-8018-158f858f80eb</t>
         </is>
       </c>
@@ -2237,6 +2759,11 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
           <t>urn:uuid:e7ea316d-6cc8-4ad9-b9d7-a519acaaaf0c</t>
         </is>
       </c>
@@ -2254,6 +2781,11 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>urn:uuid:00198fc7-790c-49da-90d7-e93e42ef82cc</t>
         </is>
       </c>
@@ -2281,6 +2813,11 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
           <t>urn:uuid:58a6eb93-dda2-46e1-9246-7d42f20557b0</t>
         </is>
       </c>
@@ -2293,6 +2830,11 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
           <t>urn:uuid:07d4d12f-47b6-4c04-9546-b28faf40c814</t>
         </is>
       </c>
@@ -2320,6 +2862,11 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
           <t>urn:uuid:17f2bd9e-1757-4087-88a4-9b74a805e23d</t>
         </is>
       </c>
@@ -2347,6 +2894,11 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
           <t>urn:uuid:b311531a-d29f-4e0e-89f0-1f8341334eae</t>
         </is>
       </c>
@@ -2359,6 +2911,11 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
           <t>urn:uuid:f7d05446-f36a-426c-a9d5-f70f558fe795</t>
         </is>
       </c>
@@ -2381,6 +2938,11 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
           <t>urn:uuid:82250dfa-1952-4cbe-ac32-3b510d49503b</t>
         </is>
       </c>
@@ -2393,6 +2955,11 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
           <t>urn:uuid:80c37523-2be3-492c-b6df-b238bf958a79</t>
         </is>
       </c>
@@ -2420,6 +2987,11 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
           <t>urn:uuid:47a4f062-e7eb-4eae-8f53-6945995d6ddc</t>
         </is>
       </c>
@@ -2432,6 +3004,11 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
           <t>urn:uuid:44a289a7-8f9a-409d-9b97-f1c2d2245c52</t>
         </is>
       </c>
@@ -2444,6 +3021,11 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
           <t>urn:uuid:2d13ab69-1389-4d45-8aa2-271deba052a7</t>
         </is>
       </c>
@@ -2456,6 +3038,11 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
           <t>urn:uuid:01443e30-96fd-431f-ad31-67619f80c12c</t>
         </is>
       </c>
@@ -2478,6 +3065,11 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
           <t>urn:uuid:adaab904-a46a-41a2-97dc-66c701d1a1fc</t>
         </is>
       </c>
@@ -2490,6 +3082,11 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
           <t>urn:uuid:f175888f-0793-4656-9ba0-60b446c40ed8</t>
         </is>
       </c>
@@ -2502,6 +3099,11 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
+          <t>unreviewed</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
           <t>urn:uuid:edf729c1-2c87-4b6b-82a2-ffecb4a95be3</t>
         </is>
       </c>
@@ -2528,6 +3130,11 @@
         </is>
       </c>
       <c r="E83" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
         <is>
           <t>urn:uuid:becca3d0-9aea-4f60-9cff-895add564144</t>
         </is>

</xml_diff>

<commit_message>
Finalize SOSA-2023 class mapping decisions
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -391,7 +391,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">

</xml_diff>

<commit_message>
Finalize SOSA-2023 object-property mapping decisions
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -1414,12 +1414,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>The chain bfo:bearer_of o cco:is_subject_of concludes in an Information Content Entity, whereas the SOSA-next relation ranges over OperatingConditions, Observation, or ObservationCollection. The chain does not express the source relation.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasOperatingConditions relates a System to OperatingConditions represented as an Observation or ObservationCollection describing conditions under which the System can operate. CCO described-by and is-subject-of expect an Information Content Entity as the describing object, while the SOSA target is an Observation or ObservationCollection. CCO capability relations instead point to an Agent Capability itself. No reviewed direct relation expresses this System-to-observational-description pattern.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>The chain bfo:bearer_of o cco:is_subject_of concludes in an Information Content Entity, whereas the SOSA-next relation ranges over Observation or ObservationCollection. The chain does not express the source relation.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. Despite its name, sosa:hasSystemCapability relates a System to an Observation or ObservationCollection describing the system's capability, not directly to the capability bearer entity. CCO has capability points from an Agent to an Agent Capability, while described-by and is-subject-of require an Information Content Entity as the description. Neither matches the SOSA observational-description pattern, and no other reviewed direct relation does so.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1614,12 +1614,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>The source relation has an Actuator subject, whereas bfo:has_participant has a process domain. The current subproperty axiom can therefore classify an actuator as a process.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:actsOn is a capability-level relation from an Actuator to a Property whose state the actuator may change. BFO/CCO process relations such as has participant and affects require a Process subject, while CCO capability and disposition relations connect a bearer to an Agent Capability or Disposition rather than to the Property that capability concerns. None therefore provides a sound superproperty for the SOSA relation.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1636,12 +1636,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>cco:affects has a continuant range, whereas sosa:Property includes the ProcessProfile branch. The current mapping can therefore impose continuant typing on an occurrent property.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:actsOnProperty relates an Actuation to a sosa:Property. The governed sosa:Property extension includes both specifically dependent continuants and ProcessProfiles. CCO affects requires an Independent Continuant target, and the reviewed participation and information relations likewise do not uniformly cover both SOSA Property branches. A direct superproperty would therefore impose unsupported typing.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1766,12 +1766,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Remove the cco:is_output_of superproperty. The source relation runs from a FeatureOfInterest to an ultimate Sample or SampleCollection. It does not relate a Continuant output to the Sampling process that produced it. The current mapping would instead place the source and target into the CCO output-to-process signature.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:featureHasUltimateSample relates an ultimate FeatureOfInterest to a Sample or SampleCollection intended to represent it. CCO represented-by requires a Representational Information Content Entity, whereas a SOSA Sample is not thereby such an information content entity. CCO output relations instead relate an output to the Sampling Process that produced it, not to the represented feature. No reviewed direct BFO/CCO relation captures the source representation relation.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1788,12 +1788,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The chain cco:described_by o cco:is_about captures an entity being described by information that is about a property. It does not establish that the entity acts on or observes that property, which is the intended meaning of sosa:forProperty. This semantic mismatch applies regardless of the CCO version.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:forProperty relates a Procedure or System to a Property that it acts on or observes. CCO aboutness and descriptive relations concern Information Content Entities, capability and disposition relations relate bearers to realizable entities, and process participation or affect relations have incompatible signatures. The previously proposed cco:described_by o cco:is_about chain also does not entail the source acts-on-or-observes semantics.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Remove the cco:has_input superproperty. The source relation runs from a Procedure, which is mapped as a prescriptive information content entity, whereas CCO has_input has a Process domain. No direct CCO superproperty expresses a Procedure-to-required-input-specification relation.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasInput relates a Procedure, governed as a prescriptive Information Content Entity, to an input required for its execution. CCO has input instead has a Process subject and encodes an Independent Continuant whose presence is necessary for process initiation. CCO requires relates a Process Regulation to a Process, and prescribes does not identify an entity as an execution input. No reviewed target relation expresses the source relation directly.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Remove the cco:has_input superproperty. Although the source subject is an Execution or ExecutionCollection, SOSA only states that the object assigns a value to an input used in the execution. It does not entail the stronger CCO condition that the object is a Continuant whose presence at the beginning is necessary for the Process to start.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasInputValue assigns a value to a Procedure-defined input used in an Execution or ExecutionCollection. CCO has input entails the stronger condition that an Independent Continuant is present at the beginning of a Process and is necessary for that Process to start. SOSA does not entail those conditions merely from an assigned input value, and no other reviewed BFO/CCO relation captures the value-assignment semantics.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1920,12 +1920,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Remove the cco:is_output_of superproperty. The source relation runs from one Sample to another Sample identified as its original. It does not relate an output to the Sampling process that produced it, and the CCO mapping would incorrectly type the target Sample as a Process.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasOriginalSample relates a Sample or SampleCollection to the initial Sample collected from the ultimate FeatureOfInterest. CCO output relations require a Process argument and therefore have the wrong signature. CCO predecessor/successor semantics require an input-output transition through a process and are stronger than the SOSA relation, which may identify the original sample across a downstream sample chain. No reviewed direct relation safely generalizes the source relation.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Remove the cco:is_output_of superproperty. The source relation runs from a Procedure to an output specification, while is_output_of runs from a Continuant output to the Process that produced it. A Procedure is not that process, and the current mapping also reverses the relation.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasOutput relates a Procedure to an output of its execution. CCO has output instead has a Process subject and requires an Independent Continuant whose presence at the end is necessary for process completion; cco:is_output_of has the opposite direction. CCO prescription relations do not entail that the related entity is an output. No reviewed direct BFO/CCO relation preserves the source semantics.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Remove the active BFO role-realization property-chain mapping. Although bfo:bearer_of o bfo:has_realization o bfo:has_participant is a valid OWL property chain, it can conclude sosa:hosts for arbitrary participants in a realization, which is broader than the SOSA hosts relation. Retain the native SOSA hosts semantics without a direct BFO/CCO mapping.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hosts relates a Platform to an Asset hosted or mounted on it. BFO located-in/location-of encode spatial containment, which is not entailed by all hosting or mounting arrangements; BFO parthood is likewise not required, and process participation does not express hosting. The previously considered role-realization chain overgenerates hosts for arbitrary participants in a realization. No reviewed direct BFO/CCO relation preserves the source semantics.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2754,12 +2754,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>cco:has_input has a continuant range, whereas sosa:Property includes the ProcessProfile branch. The current mapping can impose continuant typing on an occurrent property.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:observedProperty relates an Observation or ObservationCollection to the Property observed. CCO has input requires an Independent Continuant input whose presence at the beginning is necessary for a Process to start, which is not entailed by observation and does not cover the ProcessProfile branch of sosa:Property. CCO aboutness relations instead require an Information Content Entity subject. No reviewed BFO/CCO relation provides the required uniform semantics.</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2776,12 +2776,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>The source relation has a Sensor subject, whereas bfo:has_participant has a process domain. The current subproperty axiom can therefore classify a sensor as a process.</t>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:observes is a capability-level relation from a Sensor to a Property that the sensor is capable of sensing. BFO/CCO process relations require a Process subject, while CCO capability and disposition relations relate a bearer to an Agent Capability or Disposition rather than to the Property that capability concerns. No reviewed BFO/CCO relation preserves the SOSA semantics and signature.</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">

</xml_diff>

<commit_message>
Materialize SOSA-2023 inverse-derived mappings
Explicitly materialize nine mappings entailed through declared SOSA and BFO/CCO inverse-property pairs.

Regenerate maintained products, synchronize formal release evidence and documentation, and preserve current-track ontology bytes.
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -2192,9 +2192,24 @@
           <t>sosa:inDeployment</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>bfo:participates_in</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:inDeployment owl:inverseOf sosa:deployedOnPlatform; the governed COMS mapping asserts sosa:deployedOnPlatform rdfs:subPropertyOf bfo:has_participant; and the pinned BFO/CCO target declares bfo:has_participant owl:inverseOf bfo:participates_in. Therefore sosa:inDeployment rdfs:subPropertyOf bfo:participates_in is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2260,9 +2275,24 @@
           <t>sosa:isDetectedBy</t>
         </is>
       </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>cco:affects</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:isDetectedBy owl:inverseOf sosa:detects; the governed COMS mapping asserts sosa:detects rdfs:subPropertyOf cco:is_affected_by; and the pinned BFO/CCO target declares cco:is_affected_by owl:inverseOf cco:affects. Therefore sosa:isDetectedBy rdfs:subPropertyOf cco:affects is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2413,9 +2443,24 @@
           <t>sosa:isResultOf</t>
         </is>
       </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>cco:is_output_of</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:isResultOf owl:inverseOf sosa:hasResult; the governed COMS mapping asserts sosa:hasResult rdfs:subPropertyOf cco:has_output; and the pinned BFO/CCO target declares cco:has_output owl:inverseOf cco:is_output_of. Therefore sosa:isResultOf rdfs:subPropertyOf cco:is_output_of is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2498,9 +2543,24 @@
           <t>sosa:isSubSystemOf</t>
         </is>
       </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>bfo:continuant_part_of</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:isSubSystemOf owl:inverseOf sosa:hasSubSystem; the governed COMS mapping asserts sosa:hasSubSystem rdfs:subPropertyOf bfo:has_continuant_part; and the pinned BFO/CCO target declares bfo:has_continuant_part owl:inverseOf bfo:continuant_part_of. Therefore sosa:isSubSystemOf rdfs:subPropertyOf bfo:continuant_part_of is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2667,9 +2727,24 @@
           <t>sosa:madeExecution</t>
         </is>
       </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>cco:agent_in</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:madeExecution owl:inverseOf sosa:madeBySystem; the governed COMS mapping asserts sosa:madeBySystem rdfs:subPropertyOf cco:has_agent; and the pinned BFO/CCO target declares cco:has_agent owl:inverseOf cco:agent_in. Therefore sosa:madeExecution rdfs:subPropertyOf cco:agent_in is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2684,9 +2759,24 @@
           <t>sosa:madeObservation</t>
         </is>
       </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>cco:agent_in</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:madeObservation owl:inverseOf sosa:madeBySensor; the governed COMS mapping asserts sosa:madeBySensor rdfs:subPropertyOf cco:has_agent; and the pinned BFO/CCO target declares cco:has_agent owl:inverseOf cco:agent_in. Therefore sosa:madeObservation rdfs:subPropertyOf cco:agent_in is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2701,9 +2791,24 @@
           <t>sosa:madeSampling</t>
         </is>
       </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>cco:agent_in</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:madeSampling owl:inverseOf sosa:madeBySampler; the governed COMS mapping asserts sosa:madeBySampler rdfs:subPropertyOf cco:has_agent; and the pinned BFO/CCO target declares cco:has_agent owl:inverseOf cco:agent_in. Therefore sosa:madeSampling rdfs:subPropertyOf cco:agent_in is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3002,9 +3107,24 @@
           <t>sosa:systemDeployment</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>bfo:participates_in</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:systemDeployment owl:inverseOf sosa:deployedSystem; the governed COMS mapping asserts sosa:deployedSystem rdfs:subPropertyOf bfo:has_participant; and the pinned BFO/CCO target declares bfo:has_participant owl:inverseOf bfo:participates_in. Therefore sosa:systemDeployment rdfs:subPropertyOf bfo:participates_in is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3019,9 +3139,24 @@
           <t>sosa:usedForExecution</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>rdfs:subPropertyOf</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>cco:prescribes</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Explicit inverse-derived mapping. The pinned SOSA source declares sosa:usedForExecution owl:inverseOf sosa:usedProcedure; the governed COMS mapping asserts sosa:usedProcedure rdfs:subPropertyOf cco:prescribed_by; and the pinned BFO/CCO target declares cco:prescribed_by owl:inverseOf cco:prescribes. Therefore sosa:usedForExecution rdfs:subPropertyOf cco:prescribes is entailed. The direct COMS axiom is materialized explicitly under the project policy for inverse-derived mappings.</t>
+        </is>
+      </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>active</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">

</xml_diff>

<commit_message>
Complete SOSA-2023 mapping review
Finalize all 39 previously unreviewed governed rows as reviewed no-direct-mapping decisions with explicit semantic rationales.

Leave the four datatype-property mappings deferred, preserve all 55 active mapping axioms and maintained ontology bytes, and synchronize validation and product contracts.
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -1138,9 +1138,14 @@
           <t>sosa:NormalOperatingConditions</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO class mapping is adopted. Despite its label, sosa:NormalOperatingConditions denotes a type of Observation or ObservationCollection that describes conditions under which a system is expected to operate normally; it does not denote the environmental condition, quality, stasis, or operating range itself. CCO Nominal Stasis and related condition-oriented classes therefore have the wrong ontological category, and no reviewed BFO/CCO class directly captures this specialized SOSA observation type.</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1155,9 +1160,14 @@
           <t>sosa:OperatingConditions</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO class mapping is adopted. sosa:OperatingConditions denotes a type of Observation or ObservationCollection that describes operating conditions of systems, rather than the operating conditions themselves. Candidate BFO/CCO environmental, quality, stasis, and specification classes consequently classify different kinds of entities. Performance Specification is prescriptive information content, whereas the SOSA class consists of observational records of conditions. No reviewed target class preserves the source semantics.</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1172,9 +1182,14 @@
           <t>sosa:SuboptimalOperatingConditions</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO class mapping is adopted. sosa:SuboptimalOperatingConditions denotes a type of Observation or ObservationCollection describing conditions under which a system is expected to operate sub-optimally; it does not denote the adverse condition, degraded quality, stasis, or performance state itself. The reviewed BFO/CCO condition-oriented candidates therefore have the wrong ontological category. Its subclass relationship to sosa:OperatingConditions does not independently justify a target mapping.</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1189,9 +1204,14 @@
           <t>sosa:SurvivableConditions</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO class mapping is adopted. sosa:SurvivableConditions denotes a type of Observation or ObservationCollection describing the conditions under which a system is expected to remain physically serviceable or survive; it does not itself denote the environmental condition, survival state, quality, or stasis. The reviewed BFO/CCO condition and stasis classes therefore classify different entities, and the source subclass relationship does not independently establish a direct target mapping.</t>
+        </is>
+      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1456,9 +1476,14 @@
           <t>sosa:hasValidityContext</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasValidityContext links an Observation, ObservationCollection, or Property to an Observation or ObservationCollection that describes the context in which the former is valid. CCO describes_condition and condition_described_by require a Performance Specification and encode a specific prescriptive condition relation; organizational-context relations have unrelated agent/role semantics. The SOSA relation does not entail those conditions, and no reviewed BFO/CCO relation directly captures its observational validity-context semantics.</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1473,9 +1498,14 @@
           <t>sampling:hasSampleRelationship</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sampling:hasSampleRelationship links a SOSA Sample to a reified sampling:SampleRelationship resource that records a relationship in the SOSA Sampling model. The reviewed BFO/CCO relations express aboutness, affiliation, parthood, dependence, participation, or other substantive ontological relations rather than this model-specific link to a relationship-description resource. No reviewed target relation preserves the source relata and semantics.</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1490,9 +1520,14 @@
           <t>sampling:natureOfRelationship</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sampling:natureOfRelationship links a reified SampleRelationship to an indication of its RelationshipNature. The source relation does not entail that the nature indicator is an Information Content Entity, measurement, description, or specifically dependent continuant of the relationship. CCO descriptive, measurement, aboutness, and BFO dependence relations therefore impose unsupported typing or stronger semantics.</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1507,9 +1542,14 @@
           <t>sampling:relatedSample</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sampling:relatedSample links a reified SampleRelationship resource to the related SOSA Sample. This is a structural relation in the SOSA Sampling relationship model rather than an assertion that the SampleRelationship is an Information Content Entity about the Sample, a process involving it, or a realizable entity realized by it. The reviewed BFO/CCO candidates therefore have incompatible relata or semantic commitments.</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1840,9 +1880,14 @@
           <t>sosa:hasFeatureOfInterest</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasFeatureOfInterest is a polymorphic subject relation from an Execution or Deployment to its FeatureOfInterest: depending on the source subtype, the feature may be observed, acted on, sampled, or targeted by a deployment. BFO participation is not entailed for all such features, CCO process-object relations impose stronger conditions, and CCO aboutness requires an Information Content Entity subject. No single reviewed target relation uniformly captures the source semantics.</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1901,9 +1946,14 @@
           <t>sosa:hasMember</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasMember is a uniform SOSA collection-membership relation across collections whose members may be continuants or occurrents. BFO member parthood is restricted to material entities, while BFO occurrent parthood applies to occurrents; the continuant and occurrent parthood relations therefore cannot provide one uniform superproperty for all SOSA collection kinds. SOSA membership is retained without collapsing it into BFO parthood.</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1962,9 +2012,14 @@
           <t>sosa:hasProcedure</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasProcedure relates a Property to a Procedure that can observe or act on it. CCO prescribed_by instead asserts that the Procedure serves as a rule, guide, or model for the related entity; mere applicability of a Procedure to observing or acting on a Property does not entail that prescription relation. The source relation is also a specialization of sosa:propertyFor, for which no direct BFO/CCO mapping is adopted.</t>
+        </is>
+      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1979,9 +2034,14 @@
           <t>sosa:hasProperty</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasProperty relates a FeatureOfInterest to a sosa:Property. The governed sosa:Property extension includes both specifically dependent continuants and ProcessProfiles. BFO bearer_of applies only to specifically dependent continuants, and aggregate-bearer relations are likewise category-specific. A uniform subproperty mapping would therefore impose unsupported continuant typing on the ProcessProfile branch.</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1996,9 +2056,14 @@
           <t>sosa:hasProxy</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasProxy relates a Property to a Stimulus serving as its proxy. CCO represented_by requires the proxy relatum to be a Representational Information Content Entity, whereas a SOSA Stimulus is not thereby an Information Content Entity. CCO aboutness and descriptive relations impose the same information-content category mismatch. No reviewed direct target relation captures the proxy semantics.</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2045,9 +2110,14 @@
           <t>sosa:hasSample</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasSample relates a FeatureOfInterest to a Sample or SampleCollection intended to represent it. CCO represented_by requires a Representational Information Content Entity as the representing relatum, whereas a SOSA Sample or SampleCollection is not thereby such an information content entity. The source representative-sampling relation therefore has no reviewed direct BFO/CCO superproperty.</t>
+        </is>
+      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2089,9 +2159,14 @@
           <t>sosa:hasUltimateFeatureOfInterest</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:hasUltimateFeatureOfInterest relates an Execution, ExecutionCollection, or Deployment to its ultimate subject entity. The relation covers observation, actuation, sampling, and deployment cases with different underlying semantics. CCO aboutness requires an Information Content Entity subject, participation is not entailed for every ultimate subject, and agentive process-object relations are too strong. No single reviewed target relation uniformly captures the source relation.</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2224,9 +2299,14 @@
           <t>sosa:inputFor</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:inputFor relates an input to a Procedure that uses it in an Execution. Reversing sosa:hasInput does not remove the target mismatch: the inverse of CCO has input relates an input to a Process and inherits the stronger requirement that the input be present and necessary for process initiation, whereas the SOSA range is a Procedure, governed as a prescriptive Information Content Entity. No reviewed target relation expresses the source relation directly.</t>
+        </is>
+      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2241,9 +2321,14 @@
           <t>sosa:inputValueForExecution</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:inputValueForExecution relates an input value to an Execution that used it. The inverse of CCO has input has the broad input-to-Process direction, but it still entails that an Independent Continuant is present at the beginning and necessary for the Process to start. SOSA usage of an assigned input value does not entail those conditions, and no other reviewed relation captures the value-use semantics.</t>
+        </is>
+      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2258,9 +2343,14 @@
           <t>sosa:isActedOnBy</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isActedOnBy is a capability-level relation from a Property to an Actuator that may change its state. Reversing process relations such as affects yields a relation to a Process rather than to an Actuator, while capability and disposition relations connect a bearer to a realizable entity rather than a Property to the bearer whose capability concerns it. No reviewed target relation preserves the source semantics and signature.</t>
+        </is>
+      </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2307,9 +2397,14 @@
           <t>sosa:isFeatureOfInterestOf</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isFeatureOfInterestOf is the inverse polymorphic relation from a FeatureOfInterest to an Execution, ExecutionCollection, or Deployment for which it is the subject. Reversing participation, process-object, or aboutness candidates does not remove their unsupported participation, agentive-object, or Information Content Entity conditions. No reviewed target relation uniformly captures the source semantics.</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2324,9 +2419,14 @@
           <t>sosa:isHostedBy</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isHostedBy relates an Asset to a Platform on which it is hosted or mounted. Reversing the previously considered spatial or parthood relations does not remove their excess strength: hosting or mounting does not entail spatial containment or parthood. Process participation likewise does not express hosting. No reviewed direct BFO/CCO relation preserves the source semantics.</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2341,9 +2441,14 @@
           <t>sosa:isMemberOf</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isMemberOf is the inverse of the uniform SOSA collection-membership relation. BFO member-part-of is restricted to material entities and BFO occurrent-part-of is restricted to occurrents, so neither relation uniformly covers members of all SOSA collection types. Reversing direction does not remove the continuant/occurrent category split.</t>
+        </is>
+      </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2358,9 +2463,14 @@
           <t>sosa:isObservedBy</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isObservedBy is a capability-level relation from a Property to a Sensor able to observe it. Reversing BFO/CCO process relations still produces a Process relatum rather than a Sensor, while capability and disposition relations do not relate the Property being sensed to the bearer of the capability. No reviewed BFO/CCO relation preserves the SOSA semantics and signature.</t>
+        </is>
+      </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2375,9 +2485,14 @@
           <t>sosa:isOriginalSampleOf</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isOriginalSampleOf relates the initial Sample collected from the ultimate FeatureOfInterest to a downstream Sample or SampleCollection. Reversing CCO predecessor/successor relations does not remove their stronger requirement for an input-output transition through a Process, and output relations themselves require a Process argument. No reviewed direct relation safely generalizes the SOSA sample-chain semantics.</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2392,9 +2507,14 @@
           <t>sosa:isProcedureFor</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isProcedureFor relates a Procedure to a Property that it can observe or act on. CCO prescribes is stronger: it requires the Information Content Entity to serve as a rule, guide, or model for the related entity. A Procedure being applicable to observation or actuation of a Property does not entail that the Procedure prescribes the Property. The source relation is also a specialization of sosa:forProperty, for which no direct mapping is adopted.</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2409,9 +2529,14 @@
           <t>sosa:isPropertyOf</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isPropertyOf relates a sosa:Property to its FeatureOfInterest. Although BFO inheres_in is appropriate for specifically dependent continuants, the governed sosa:Property extension also includes ProcessProfiles, which are occurrent-side entities and do not inhere in a bearer. No reviewed target relation uniformly covers both branches of the source class.</t>
+        </is>
+      </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2426,9 +2551,14 @@
           <t>sosa:isProxyFor</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isProxyFor relates a Stimulus to the Property for which it serves as proxy. CCO represents requires a Representational Information Content Entity subject, and CCO is_about requires an Information Content Entity subject. A SOSA Stimulus is not thereby either kind of information content entity, so the apparent representation candidates have incompatible typing.</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2475,9 +2605,14 @@
           <t>sosa:isResultOfMadeBySampler</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isResultOfMadeBySampler is a mediated shortcut from a Sample or SampleCollection to the Sampler that made the Sampling whose result it is. CCO is_output_of relates an output to the producing Process, not to the Process's Agent, while has_agent/agent_in relate an Agent to that Process rather than directly to its output. The SOSA shortcut therefore corresponds to a composition of relations, not to a reviewed primitive BFO/CCO object property.</t>
+        </is>
+      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2492,9 +2627,14 @@
           <t>sosa:isResultOfUsedProcedure</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isResultOfUsedProcedure is a mediated shortcut from a Sample or SampleCollection to the SamplingProcedure used in the Sampling that produced it. CCO is_output_of relates the output to the Process, not to the prescriptive Procedure, while prescribed_by relates an Entity to a prescribing Information Content Entity without entailing that the entity is a result produced through its use. No reviewed primitive target relation captures the composed semantics.</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2509,9 +2649,14 @@
           <t>sosa:isSampleOf</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isSampleOf relates a Sample or SampleCollection to the FeatureOfInterest it is intended to represent. CCO represents requires a Representational Information Content Entity subject, which is not entailed for SOSA Samples. The source sampling/representative relation therefore cannot safely be generalized by the reviewed CCO representation relations.</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2526,9 +2671,14 @@
           <t>sosa:isSampleOfUltimateFOI</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isSampleOfUltimateFOI relates a Sample or SampleCollection to the ultimate FeatureOfInterest that it is intended to be representative of. Reversing CCO representation relations does not remove the typing mismatch because a SOSA Sample is not thereby a Representational Information Content Entity. CCO output relations instead concern the Sampling Process that produced an output, not the represented feature. No reviewed direct relation captures the source semantics.</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2575,9 +2725,14 @@
           <t>sosa:isUltimateFeatureOfInterestOf</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:isUltimateFeatureOfInterestOf is the inverse relation from an ultimate FeatureOfInterest to an Execution, ExecutionCollection, or Deployment for which it is the ultimate subject. Reversing CCO aboutness, participation, or process-object candidates preserves their incompatible typing or stronger semantic conditions. No reviewed target relation uniformly captures the source relation.</t>
+        </is>
+      </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2823,9 +2978,14 @@
           <t>sosa:madeSamplingHasResult</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:madeSamplingHasResult is a mediated shortcut from a Sampler to the Sample or SampleCollection resulting from a Sampling made by that Sampler. CCO agent_in relates the Sampler to the Sampling Process and CCO has_output relates the Process to its output, but neither relation directly relates the Agent to the output. No reviewed primitive BFO/CCO relation expresses the composed source semantics.</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2840,9 +3000,14 @@
           <t>sosa:observationRelatedTo</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:observationRelatedTo deliberately expresses broad relatedness from an Observation or ObservationCollection to another Execution or ExecutionCollection. The source relation can cover different bases of relatedness rather than one fixed ontological relation. CCO aboutness requires an Information Content Entity subject and other reviewed process relations impose specific causal, parthood, participation, or realization semantics not entailed by SOSA. No single reviewed target relation captures this generic relatedness.</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2933,9 +3098,14 @@
           <t>sosa:outputFor</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:outputFor relates an output to a Procedure that generates it in an Execution. Although cco:is_output_of has the same broad direction, it relates an output to a Process and carries the CCO process-output conditions; the SOSA range is instead a Procedure, governed as a prescriptive Information Content Entity. Reversing direction therefore does not repair the signature mismatch, and no reviewed direct relation preserves the source semantics.</t>
+        </is>
+      </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3014,9 +3184,14 @@
           <t>sosa:propertyFor</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:propertyFor relates a Property to a Procedure or System that acts on it or observes it. Reversing CCO aboutness or descriptive relations still yields information-content semantics rather than the source acts-on-or-observes relation, and capability, disposition, participation, and affect relations have incompatible signatures. No reviewed direct BFO/CCO relation expresses the source relation.</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3058,9 +3233,14 @@
           <t>sosa:relatedObservation</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:relatedObservation is the inverse broad-relatedness relation from an Execution or ExecutionCollection to an Observation or ObservationCollection. Reversing aboutness or other specific process relations does not eliminate their unsupported information-content, causal, parthood, participation, or realization commitments. No single reviewed target relation captures the intentionally generic source semantics.</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3171,9 +3351,14 @@
           <t>sosa:usedForExecutionHasResult</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:usedForExecutionHasResult is a mediated shortcut from a SamplingProcedure to a Sample or SampleCollection resulting from an Execution that used the Procedure. CCO prescribes can relate the Procedure to the Process and CCO has_output can relate the Process to its output, but use of a Procedure does not entail that the Procedure directly prescribes that particular output. No reviewed primitive target relation captures the composed source semantics.</t>
+        </is>
+      </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3215,9 +3400,14 @@
           <t>sosa:wasActedOnBy</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:wasActedOnBy relates a Property to an Actuation that changed its state. Reversing CCO affects would require the affected relatum to satisfy the corresponding Independent Continuant typing, but the governed sosa:Property extension includes both specifically dependent continuants and ProcessProfiles. The same unsupported typing therefore remains in the inverse direction, and no reviewed relation uniformly captures the source semantics.</t>
+        </is>
+      </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3232,9 +3422,14 @@
           <t>sosa:wasObservedBy</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>No direct BFO/CCO object-property mapping is adopted. sosa:wasObservedBy relates a Property to an Observation that observed it. Reversing CCO has input would give the broad Property-to-Process direction but retains the stronger necessary-at-process-start condition and Independent Continuant typing, which does not cover the ProcessProfile branch of sosa:Property. Reversed aboutness relations instead impose Information Content Entity semantics. No reviewed BFO/CCO relation provides the required uniform semantics.</t>
+        </is>
+      </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>unreviewed</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">

</xml_diff>

<commit_message>
Finalize SOSA-2023 datatype-property decisions
Review the four remaining SOSA datatype properties against the pinned BFO/CCO target and finalize each as no_direct_mapping.

The target provides only narrower datatype-specific value properties, so no direct mapping is sound; all 119 governed mapping decisions are now final while active ontology products remain byte-identical.
</commit_message>
<xml_diff>
--- a/mappings/SOSA-next-to-BFO-COMS.xlsx
+++ b/mappings/SOSA-next-to-BFO-COMS.xlsx
@@ -1566,12 +1566,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Datatype-property mapping deferred pending repository-wide COMS support for datatype-property source terms. This capability must be implemented consistently for both the current SOSA mapping and the forthcoming SOSA mapping.</t>
+          <t>No direct BFO/CCO datatype-property mapping is adopted. sosa:endTime permits temporal literal values across the SOSA temporal value space, including xsd:dateTime, xsd:date, xsd:gYearMonth, and xsd:gYear. The pinned CCO target instead provides datatype-specific properties such as has datetime value and has date value. Each candidate is narrower than the SOSA value space, so asserting a subproperty mapping would impose an unsupported datatype constraint. No reviewed generic CCO temporal-value datatype property preserves the source semantics.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1588,12 +1588,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Datatype-property mapping deferred pending repository-wide COMS support for datatype-property source terms. This capability must be implemented consistently for both the current SOSA mapping and the forthcoming SOSA mapping.</t>
+          <t>No direct BFO/CCO datatype-property mapping is adopted. sosa:hasSimpleResult permits an Execution result to be represented directly by a literal without requiring one fixed literal datatype. The pinned CCO target provides separate datatype-specific value properties such as has text value, has decimal value, has boolean value, has integer value, has double value, and has datetime value. Mapping SOSA hasSimpleResult to any one of these would incorrectly restrict otherwise valid SOSA results, and no reviewed generic CCO literal-value datatype property captures the source relation.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Datatype-property mapping deferred pending repository-wide COMS support for datatype-property source terms. This capability must be implemented consistently for both the current SOSA mapping and the forthcoming SOSA mapping.</t>
+          <t>No direct BFO/CCO datatype-property mapping is adopted. sosa:resultTime permits temporal literal values across the SOSA temporal value space, including xsd:dateTime, xsd:date, xsd:gYearMonth, and xsd:gYear. The pinned CCO has datetime value and has date value properties each constrain the value to a narrower datatype and therefore cannot soundly generalize the full SOSA relation. No reviewed generic CCO temporal-value datatype property preserves the source semantics.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1632,12 +1632,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Datatype-property mapping deferred pending repository-wide COMS support for datatype-property source terms. This capability must be implemented consistently for both the current SOSA mapping and the forthcoming SOSA mapping.</t>
+          <t>No direct BFO/CCO datatype-property mapping is adopted. sosa:startTime permits temporal literal values across the SOSA temporal value space, including xsd:dateTime, xsd:date, xsd:gYearMonth, and xsd:gYear. The pinned CCO target instead provides narrower datatype-specific properties such as has datetime value and has date value. A direct subproperty mapping would therefore impose unsupported datatype constraints on valid SOSA values. No reviewed generic CCO temporal-value datatype property preserves the source semantics.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>no_direct_mapping</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">

</xml_diff>